<commit_message>
Update JINZZA_todo.xlsx to reflect 2026-09-08 work
Marked 38 rows done/updated across planning, lobby, round logic, sound,
UI/UX, and props based on this session's actual changes (kiosk placement,
Customization/EmoteWheel widget trees, Question Time cycles setting, dead
UI cleanup, TEMP audio hooks, and the commit/push itself). Recomputed the
summary sheet's per-category and overall totals to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KbsqpAAUuew2ZVxs2nwomV
</commit_message>
<xml_diff>
--- a/docs/JINZZA_todo.xlsx
+++ b/docs/JINZZA_todo.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="448">
   <si>
     <t xml:space="preserve">No</t>
   </si>
@@ -11236,6 +11236,120 @@
   </si>
   <si>
     <t xml:space="preserve">전체 합계</t>
+  </si>
+  <si>
+    <t>조작 탭의 Shoot/SwapWeapon 리바인드 행 제거 완료 - IA_Shoot/IA_SwapWeapon은 AjinzzaCharacter가 바인딩하지 않는 죽은 UI였음 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>origin(https://github.com/KINGWONWOO/jinzza)에 커밋 및 push 완료 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>Lvl_Lobby에 배치 완료(-400,0,80), 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>Lvl_Lobby에 배치 완료(400,0,80), 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>EnterKioskUIMode/ExitKioskUIMode로 수정, 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>UjinzzaCustomizationWidget에 실제 BuildWidgetTree 구현(5개 항목 Prev/Next + Done), AjinzzaWardrobeKiosk를 (0,400,80)에 배치, 메인메뉴 Customize 버튼도 연결, 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>UjinzzaGameUserSettings::SaveSettings()로 config 파일에 영구 저장됨 - 별도 저장 시스템 불필요 (2026-09-08 확인)</t>
+  </si>
+  <si>
+    <t>FJinzzaMatchSettings::QuestionTimeCycles(1-3) 추가, Room Settings 패널에 스핀박스 행 추가, RoundPhaseSubsystem이 65s*cycles로 계산 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>AssignRoles()의 [TEMP DEBUG] 로그 제거 완료 (2026-09-08) - PostLogin/TryStartRound 수정은 2026-09-01부터 안정적으로 확인됨</t>
+  </si>
+  <si>
+    <t>jinzzaCharacterCustomizationComponent.h/.cpp로 이미 구현되어 있었음(UjinzzaGameUserSettings 값을 캐릭터에 적용) - 시트가 최신화되지 않았던 항목, 실제 파츠 콘텐츠 없어 일부 no-op (2026-09-08 확인)</t>
+  </si>
+  <si>
+    <t>TEMP 플레이스홀더(LobbyPannelOpen.wav) 진입음 추가 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>설정 사이드바 탭 버튼이 이미 JinzzaUI::MakeSecondaryButton 공용 클릭음을 자동 재생 중 - 별도 구현 불필요 (2026-09-08 확인)</t>
+  </si>
+  <si>
+    <t>AjinzzaInteractableKiosk::EnterKioskUIMode + AjinzzaStartMatchKiosk::Interact에 TEMP 확인음(LobbyPannelOpen.wav) 추가 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>메인메뉴/키오스크 양쪽 진입 경로 모두 TEMP 플레이스홀더(LobbyPannelOpen.wav) 재생 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>Prev/Next 버튼이 이미 JinzzaUI::MakeSecondaryButton 공용 클릭음을 자동 재생 중 - 별도 구현 불필요 (2026-09-08 확인)</t>
+  </si>
+  <si>
+    <t>Client_ReceiveRoleAssignment_Implementation에 TEMP 플레이스홀더(correctanswer.wav) 추가 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>AjinzzaGameGameState::OnPhaseChanged 구독하는 신규 HandlePhaseChanged에서 TEMP 플레이스홀더(PressButton.wav) 재생 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>TEMP 플레이스홀더(PressButton.wav) 연결 및 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>TEMP 플레이스홀더(Punch1.wav) 연결 및 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>AjinzzaBoomboxProp, TEMP 플레이스홀더(FruitGameBgm) 연결 및 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>UpdateFootsteps(), 150cm 간격, Footstep/FootstepGrass 랜덤 교차 재생, 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>DoJumpStart에서 재생, 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>신규 Landed() 오버라이드, 빌드 성공 확인 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>Multicast_PlayEmote_Implementation에 TEMP 플레이스홀더(Punch1.wav) 추가, 몽타주 없어도 재생됨 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>TEMP 플레이스홀더(correctanswer.wav) 추가 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>TEMP 플레이스홀더(WrongAnswerSound.wav, 신규 이식) 추가 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>TEMP 플레이스홀더(PressButton.wav) 추가 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>TEMP으로 QuizGameBgm을 Lvl_Game 전체 BGM으로 사용 중, 빌드 성공 확인 (2026-09-08) - 추후 정식 트랙으로 교체 예정</t>
+  </si>
+  <si>
+    <t>UjinzzaEmoteWheelWidget에 BuildWidgetTree 추가 - 텍스트 십자 레이아웃으로 호버 시 하이라이트되는 실제 동작 UI 구현 완료 (구현 완료, 시안/아이콘 아트는 여전히 미정) (2026-09-08)</t>
+  </si>
+  <si>
+    <t>BP·상호작용 로직 + TEMP 사운드(PressButton.wav) 연결, 빌드 성공 확인 (2026-09-08) - 정식 메시/사운드는 추후 교체</t>
+  </si>
+  <si>
+    <t>BP·상호작용 로직 + TEMP 사운드(Punch1.wav) 연결, 빌드 성공 확인 (2026-09-08) - 정식 메시/사운드는 추후 교체</t>
+  </si>
+  <si>
+    <t>AjinzzaBoomboxProp, TEMP 사운드(FruitGameBgm) 연결, 빌드 성공 확인 (2026-09-08) - 기획서 목록과 명칭 불일치는 별도 결정 필요</t>
+  </si>
+  <si>
+    <t>TEMP 사운드(InteractWoodenBox) 연결, 빌드 성공 확인 (2026-09-08) - 기획서 8종 목록에 없는 신규 소품</t>
+  </si>
+  <si>
+    <t>AjinzzaBasketballHoop::Multicast_PlayScoreEffects, TEMP 사운드(correctanswer) 연결, 빌드 성공 확인 (2026-09-08) - 득점 이펙트(Niagara)는 별도 미구현</t>
+  </si>
+  <si>
+    <t>TEMP 사운드(Stunned) 연결, 빌드 성공 확인 (2026-09-08) - 기획서에 없는 신규 소품</t>
+  </si>
+  <si>
+    <t>AssignRoles()의 [TEMP DEBUG] 로그 제거 완료 (2026-09-08)</t>
+  </si>
+  <si>
+    <t>2026-09-08 변경사항 빌드 성공 확인됨 (unity 빌드 충돌 이슈도 해결) - 실제 플레이테스트는 아직 진행 전</t>
+  </si>
+  <si>
+    <t>origin/main에 커밋 및 push 완료 (2026-09-08) - 커밋 6265abb</t>
   </si>
 </sst>
 </file>
@@ -11793,7 +11907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -12135,10 +12249,10 @@
         <v>41</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>42</v>
+        <v>410</v>
       </c>
       <c r="G17" s="9" t="s">
         <v>12</v>
@@ -12323,10 +12437,10 @@
         <v>61</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>62</v>
+        <v>411</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>46</v>
@@ -12705,10 +12819,10 @@
         <v>104</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>106</v>
+        <v>412</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>91</v>
@@ -12724,10 +12838,10 @@
         <v>107</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>108</v>
+        <v>413</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>91</v>
@@ -12743,10 +12857,10 @@
         <v>109</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>110</v>
+        <v>414</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>91</v>
@@ -12764,10 +12878,10 @@
         <v>112</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>113</v>
+        <v>415</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>91</v>
@@ -12783,10 +12897,10 @@
         <v>114</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>115</v>
+        <v>416</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>91</v>
@@ -12950,10 +13064,10 @@
         <v>131</v>
       </c>
       <c r="E60" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>132</v>
+        <v>417</v>
       </c>
       <c r="G60" s="9" t="s">
         <v>123</v>
@@ -13233,10 +13347,10 @@
         <v>160</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>161</v>
+        <v>418</v>
       </c>
       <c r="G75" s="9" t="s">
         <v>123</v>
@@ -13400,9 +13514,11 @@
         <v>177</v>
       </c>
       <c r="E84" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F84" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F84" s="10" t="s">
+        <v>419</v>
+      </c>
       <c r="G84" s="9" t="s">
         <v>166</v>
       </c>
@@ -13694,10 +13810,10 @@
         <v>205</v>
       </c>
       <c r="E100" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F100" s="7" t="s">
-        <v>206</v>
+        <v>420</v>
       </c>
       <c r="G100" s="9" t="s">
         <v>207</v>
@@ -13751,9 +13867,11 @@
         <v>212</v>
       </c>
       <c r="E103" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F103" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F103" s="10" t="s">
+        <v>421</v>
+      </c>
       <c r="G103" s="9" t="s">
         <v>207</v>
       </c>
@@ -13768,9 +13886,11 @@
         <v>213</v>
       </c>
       <c r="E104" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F104" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F104" s="10" t="s">
+        <v>420</v>
+      </c>
       <c r="G104" s="9" t="s">
         <v>207</v>
       </c>
@@ -13785,9 +13905,11 @@
         <v>214</v>
       </c>
       <c r="E105" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F105" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F105" s="10" t="s">
+        <v>422</v>
+      </c>
       <c r="G105" s="9" t="s">
         <v>207</v>
       </c>
@@ -13802,9 +13924,11 @@
         <v>215</v>
       </c>
       <c r="E106" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F106" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F106" s="10" t="s">
+        <v>423</v>
+      </c>
       <c r="G106" s="9" t="s">
         <v>207</v>
       </c>
@@ -13819,9 +13943,11 @@
         <v>216</v>
       </c>
       <c r="E107" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F107" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F107" s="10" t="s">
+        <v>424</v>
+      </c>
       <c r="G107" s="9" t="s">
         <v>207</v>
       </c>
@@ -13836,9 +13962,11 @@
         <v>217</v>
       </c>
       <c r="E108" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F108" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F108" s="10" t="s">
+        <v>425</v>
+      </c>
       <c r="G108" s="9" t="s">
         <v>207</v>
       </c>
@@ -13853,9 +13981,11 @@
         <v>218</v>
       </c>
       <c r="E109" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F109" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F109" s="10" t="s">
+        <v>426</v>
+      </c>
       <c r="G109" s="9" t="s">
         <v>207</v>
       </c>
@@ -13974,10 +14104,10 @@
         <v>226</v>
       </c>
       <c r="E116" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F116" s="10" t="s">
-        <v>227</v>
+        <v>427</v>
       </c>
       <c r="G116" s="9" t="s">
         <v>207</v>
@@ -13993,10 +14123,10 @@
         <v>228</v>
       </c>
       <c r="E117" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F117" s="10" t="s">
-        <v>229</v>
+        <v>428</v>
       </c>
       <c r="G117" s="9" t="s">
         <v>207</v>
@@ -14107,10 +14237,10 @@
         <v>236</v>
       </c>
       <c r="E123" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F123" s="7" t="s">
-        <v>237</v>
+        <v>429</v>
       </c>
       <c r="G123" s="9" t="s">
         <v>207</v>
@@ -14128,10 +14258,10 @@
         <v>239</v>
       </c>
       <c r="E124" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F124" s="10" t="s">
-        <v>240</v>
+        <v>430</v>
       </c>
       <c r="G124" s="9" t="s">
         <v>207</v>
@@ -14147,10 +14277,10 @@
         <v>241</v>
       </c>
       <c r="E125" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F125" s="10" t="s">
-        <v>242</v>
+        <v>431</v>
       </c>
       <c r="G125" s="9" t="s">
         <v>207</v>
@@ -14166,10 +14296,10 @@
         <v>243</v>
       </c>
       <c r="E126" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F126" s="7" t="s">
-        <v>244</v>
+        <v>432</v>
       </c>
       <c r="G126" s="9" t="s">
         <v>207</v>
@@ -14187,9 +14317,11 @@
         <v>246</v>
       </c>
       <c r="E127" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F127" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F127" s="10" t="s">
+        <v>433</v>
+      </c>
       <c r="G127" s="9" t="s">
         <v>207</v>
       </c>
@@ -14204,9 +14336,11 @@
         <v>247</v>
       </c>
       <c r="E128" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F128" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F128" s="10" t="s">
+        <v>434</v>
+      </c>
       <c r="G128" s="9" t="s">
         <v>207</v>
       </c>
@@ -14221,9 +14355,11 @@
         <v>248</v>
       </c>
       <c r="E129" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F129" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F129" s="10" t="s">
+        <v>435</v>
+      </c>
       <c r="G129" s="9" t="s">
         <v>207</v>
       </c>
@@ -14238,9 +14374,11 @@
         <v>249</v>
       </c>
       <c r="E130" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F130" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F130" s="10" t="s">
+        <v>436</v>
+      </c>
       <c r="G130" s="9" t="s">
         <v>207</v>
       </c>
@@ -14295,10 +14433,10 @@
         <v>255</v>
       </c>
       <c r="E133" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F133" s="10" t="s">
-        <v>256</v>
+        <v>437</v>
       </c>
       <c r="G133" s="9" t="s">
         <v>207</v>
@@ -15113,9 +15251,11 @@
         <v>336</v>
       </c>
       <c r="E177" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F177" s="10"/>
+        <v>105</v>
+      </c>
+      <c r="F177" s="10" t="s">
+        <v>438</v>
+      </c>
       <c r="G177" s="9" t="s">
         <v>337</v>
       </c>
@@ -15149,10 +15289,10 @@
         <v>340</v>
       </c>
       <c r="E179" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F179" s="10" t="s">
-        <v>341</v>
+        <v>439</v>
       </c>
       <c r="G179" s="9" t="s">
         <v>337</v>
@@ -15168,10 +15308,10 @@
         <v>342</v>
       </c>
       <c r="E180" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F180" s="10" t="s">
-        <v>343</v>
+        <v>440</v>
       </c>
       <c r="G180" s="9" t="s">
         <v>337</v>
@@ -15282,10 +15422,10 @@
         <v>350</v>
       </c>
       <c r="E186" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F186" s="10" t="s">
-        <v>351</v>
+        <v>441</v>
       </c>
       <c r="G186" s="9" t="s">
         <v>337</v>
@@ -15322,10 +15462,10 @@
         <v>355</v>
       </c>
       <c r="E188" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F188" s="10" t="s">
-        <v>356</v>
+        <v>442</v>
       </c>
       <c r="G188" s="9" t="s">
         <v>337</v>
@@ -15341,10 +15481,10 @@
         <v>357</v>
       </c>
       <c r="E189" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F189" s="10" t="s">
-        <v>358</v>
+        <v>443</v>
       </c>
       <c r="G189" s="9" t="s">
         <v>337</v>
@@ -15360,10 +15500,10 @@
         <v>359</v>
       </c>
       <c r="E190" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F190" s="10" t="s">
-        <v>360</v>
+        <v>444</v>
       </c>
       <c r="G190" s="9" t="s">
         <v>337</v>
@@ -15533,9 +15673,11 @@
         <v>160</v>
       </c>
       <c r="E199" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F199" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="F199" s="10" t="s">
+        <v>445</v>
+      </c>
       <c r="G199" s="9" t="s">
         <v>376</v>
       </c>
@@ -15550,10 +15692,10 @@
         <v>380</v>
       </c>
       <c r="E200" s="13" t="s">
-        <v>105</v>
+        <v>10</v>
       </c>
       <c r="F200" s="7" t="s">
-        <v>381</v>
+        <v>414</v>
       </c>
       <c r="G200" s="9" t="s">
         <v>376</v>
@@ -15628,10 +15770,10 @@
         <v>389</v>
       </c>
       <c r="E204" s="11" t="s">
-        <v>29</v>
+        <v>105</v>
       </c>
       <c r="F204" s="7" t="s">
-        <v>390</v>
+        <v>446</v>
       </c>
       <c r="G204" s="9" t="s">
         <v>376</v>
@@ -15738,10 +15880,10 @@
         <v>400</v>
       </c>
       <c r="E210" s="11" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F210" s="7" t="s">
-        <v>401</v>
+        <v>447</v>
       </c>
       <c r="G210" s="9" t="s">
         <v>398</v>
@@ -15873,12 +16015,12 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing ns1:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -15916,73 +16058,73 @@
       <c r="A2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A2,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>8</v>
-      </c>
-      <c r="C2" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A2,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>0</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A2,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>8</v>
-      </c>
-      <c r="E2" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" s="4">
         <f aca="false">SUM(B2:D2)</f>
         <v>16</v>
       </c>
-      <c r="F2" s="16" t="n">
+      <c r="F2" s="16">
         <f aca="false">IF(E2=0,0,(B2+C2*0.5)/E2)</f>
-        <v>0.5</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A3,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A3,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>0</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A3,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>9</v>
-      </c>
-      <c r="E3" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="4">
         <f aca="false">SUM(B3:D3)</f>
         <v>11</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="16">
         <f aca="false">IF(E3=0,0,(B3+C3*0.5)/E3)</f>
-        <v>0.181818181818182</v>
+        <v>0.272727272727273</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A4,'작업 목록'!$E$2:$E$213,"완료")</f>
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A4,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>0</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A4,'작업 목록'!$E$2:$E$213,"예정")</f>
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="4">
         <f aca="false">SUM(B4:D4)</f>
         <v>11</v>
       </c>
-      <c r="F4" s="16" t="n">
+      <c r="F4" s="16">
         <f aca="false">IF(E4=0,0,(B4+C4*0.5)/E4)</f>
         <v>0.909090909090909</v>
       </c>
@@ -15991,173 +16133,173 @@
       <c r="A5" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A5,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>7</v>
-      </c>
-      <c r="C5" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A5,'작업 목록'!$E$2:$E$213,"부분완료")</f>
-        <v>4</v>
-      </c>
-      <c r="D5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A5,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>4</v>
-      </c>
-      <c r="E5" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4">
         <f aca="false">SUM(B5:D5)</f>
         <v>15</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="16">
         <f aca="false">IF(E5=0,0,(B5+C5*0.5)/E5)</f>
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A6,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>7</v>
-      </c>
-      <c r="C6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A6,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>1</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A6,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>13</v>
-      </c>
-      <c r="E6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4">
         <f aca="false">SUM(B6:D6)</f>
         <v>21</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="16">
         <f aca="false">IF(E6=0,0,(B6+C6*0.5)/E6)</f>
-        <v>0.357142857142857</v>
+        <v>0.428571428571429</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A7,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>2</v>
-      </c>
-      <c r="C7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A7,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>1</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A7,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>10</v>
-      </c>
-      <c r="E7" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E7" s="4">
         <f aca="false">SUM(B7:D7)</f>
         <v>13</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="16">
         <f aca="false">IF(E7=0,0,(B7+C7*0.5)/E7)</f>
-        <v>0.192307692307692</v>
+        <v>0.230769230769231</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A8,'작업 목록'!$E$2:$E$213,"완료")</f>
         <v>0</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A8,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>1</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A8,'작업 목록'!$E$2:$E$213,"예정")</f>
         <v>10</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="4">
         <f aca="false">SUM(B8:D8)</f>
         <v>11</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="16">
         <f aca="false">IF(E8=0,0,(B8+C8*0.5)/E8)</f>
-        <v>0.0454545454545455</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A9,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>8</v>
-      </c>
-      <c r="C9" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="C9" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A9,'작업 목록'!$E$2:$E$213,"부분완료")</f>
-        <v>6</v>
-      </c>
-      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A9,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>33</v>
-      </c>
-      <c r="E9" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" s="4">
         <f aca="false">SUM(B9:D9)</f>
         <v>47</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="16">
         <f aca="false">IF(E9=0,0,(B9+C9*0.5)/E9)</f>
-        <v>0.234042553191489</v>
+        <v>0.574468085106383</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A10,'작업 목록'!$E$2:$E$213,"완료")</f>
         <v>7</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A10,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A10,'작업 목록'!$E$2:$E$213,"예정")</f>
         <v>11</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="4">
         <f aca="false">SUM(B10:D10)</f>
         <v>19</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="16">
         <f aca="false">IF(E10=0,0,(B10+C10*0.5)/E10)</f>
-        <v>0.394736842105263</v>
+        <v>0.368421052631579</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A11,'작업 목록'!$E$2:$E$213,"완료")</f>
         <v>2</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A11,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>0</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A11,'작업 목록'!$E$2:$E$213,"예정")</f>
         <v>9</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="4">
         <f aca="false">SUM(B11:D11)</f>
         <v>11</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="16">
         <f aca="false">IF(E11=0,0,(B11+C11*0.5)/E11)</f>
         <v>0.181818181818182</v>
       </c>
@@ -16166,48 +16308,48 @@
       <c r="A12" s="15" t="s">
         <v>334</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A12,'작업 목록'!$E$2:$E$213,"완료")</f>
+        <v>7</v>
+      </c>
+      <c r="C12" s="4">
+        <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A12,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>1</v>
       </c>
-      <c r="C12" s="4" t="n">
-        <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A12,'작업 목록'!$E$2:$E$213,"부분완료")</f>
+      <c r="D12" s="4">
+        <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A12,'작업 목록'!$E$2:$E$213,"예정")</f>
         <v>6</v>
       </c>
-      <c r="D12" s="4" t="n">
-        <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A12,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>7</v>
-      </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="4">
         <f aca="false">SUM(B12:D12)</f>
         <v>14</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="16">
         <f aca="false">IF(E12=0,0,(B12+C12*0.5)/E12)</f>
-        <v>0.285714285714286</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
         <v>361</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A13,'작업 목록'!$E$2:$E$213,"완료")</f>
         <v>5</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A13,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>0</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A13,'작업 목록'!$E$2:$E$213,"예정")</f>
         <v>1</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="4">
         <f aca="false">SUM(B13:D13)</f>
         <v>6</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="16">
         <f aca="false">IF(E13=0,0,(B13+C13*0.5)/E13)</f>
         <v>0.833333333333333</v>
       </c>
@@ -16216,75 +16358,75 @@
       <c r="A14" s="15" t="s">
         <v>372</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A14,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>3</v>
-      </c>
-      <c r="C14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A14,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>1</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A14,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>7</v>
-      </c>
-      <c r="E14" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="4">
         <f aca="false">SUM(B14:D14)</f>
         <v>11</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="16">
         <f aca="false">IF(E14=0,0,(B14+C14*0.5)/E14)</f>
-        <v>0.318181818181818</v>
+        <v>0.454545454545455</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
         <v>395</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A15,'작업 목록'!$E$2:$E$213,"완료")</f>
-        <v>0</v>
-      </c>
-      <c r="C15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A15,'작업 목록'!$E$2:$E$213,"부분완료")</f>
         <v>0</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="4">
         <f aca="false">COUNTIFS('작업 목록'!$G$2:$G$213,A15,'작업 목록'!$E$2:$E$213,"예정")</f>
-        <v>6</v>
-      </c>
-      <c r="E15" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="4">
         <f aca="false">SUM(B15:D15)</f>
         <v>6</v>
       </c>
-      <c r="F15" s="16" t="n">
+      <c r="F15" s="16">
         <f aca="false">IF(E15=0,0,(B15+C15*0.5)/E15)</f>
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
         <v>409</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="18">
         <f aca="false">SUM(B2:B15)</f>
-        <v>62</v>
-      </c>
-      <c r="C16" s="18" t="n">
+        <v>100</v>
+      </c>
+      <c r="C16" s="18">
         <f aca="false">SUM(C2:C15)</f>
-        <v>21</v>
-      </c>
-      <c r="D16" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" s="18">
         <f aca="false">SUM(D2:D15)</f>
-        <v>129</v>
-      </c>
-      <c r="E16" s="18" t="n">
+        <v>106</v>
+      </c>
+      <c r="E16" s="18">
         <f aca="false">SUM(E2:E15)</f>
         <v>212</v>
       </c>
-      <c r="F16" s="19" t="n">
+      <c r="F16" s="19">
         <f aca="false">IF(E16=0,0,(B16+C16*0.5)/E16)</f>
-        <v>0.341981132075472</v>
+        <v>0.471698113207547</v>
       </c>
     </row>
   </sheetData>

</xml_diff>